<commit_message>
feat: confirm DPS bus fee cadence, add Pre-Nursery band, import script
Owner confirmed 2026-07-16: Bus Fee is monthly, Rs 700 (transport
students only) — resolves the "PENDING CONFIRMATION" note this file
carried since 2026-07-07. Also added a Pre-Nursery Tuition Fee row
(Rs 700, same band as Nursery-U.KG) since that class didn't exist
when the file was first built. New script runs
services.finance.import_and_generate — imports the structure and
generates the ledger for every active student atomically.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/School_docs/Daffodils/DPS_Fee_Structure_Import.xlsx
+++ b/School_docs/Daffodils/DPS_Fee_Structure_Import.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -491,7 +491,6 @@
           <t>all</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -517,7 +516,6 @@
           <t>all</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -573,7 +571,6 @@
           <t>all</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -599,7 +596,6 @@
           <t>all</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -625,7 +621,6 @@
           <t>all</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -651,7 +646,6 @@
           <t>all</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -677,7 +671,6 @@
           <t>all</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -703,7 +696,6 @@
           <t>all</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -729,7 +721,6 @@
           <t>all</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1087,7 +1078,37 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>PENDING CONFIRMATION: assumed monthly (listed alongside Monthly Fee table, and a one-month-advance note applies) -- confirm before import. If actually annual/one_time, change the Fee Type column to match.</t>
+          <t>Confirmed monthly by owner 2026-07-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Tuition Fee</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Pre-Nursery</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>700</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Pre Nursery - U.KG band per source doc</t>
         </is>
       </c>
     </row>

</xml_diff>